<commit_message>
start adding 2025 and 2026
</commit_message>
<xml_diff>
--- a/data/CV_DA_2026.xlsx
+++ b/data/CV_DA_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10421"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10303"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DA Research/Personal/CV_Build/DA_CV_2025_1/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dionne/Documents/GitHub/cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A73B5A33-5BA7-264C-B226-26824285ED69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{546A50B0-5BAE-9C42-B4E7-E7687CF18743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="61560" yWindow="-280" windowWidth="23040" windowHeight="20600" activeTab="3" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="20140" activeTab="10" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
   </bookViews>
   <sheets>
     <sheet name="positions" sheetId="11" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="other_sci_comm" sheetId="8" r:id="rId9"/>
     <sheet name="publications" sheetId="9" r:id="rId10"/>
     <sheet name="tools" sheetId="12" r:id="rId11"/>
+    <sheet name="translational" sheetId="13" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="288">
   <si>
     <t>degree</t>
   </si>
@@ -904,6 +905,12 @@
   </si>
   <si>
     <t>Mentor for two students at a high school; I supervised and taught them about malaria and public health. They wrote a project about this work.</t>
+  </si>
+  <si>
+    <t>SeroTrackR</t>
+  </si>
+  <si>
+    <t>wastewateR</t>
   </si>
 </sst>
 </file>
@@ -972,7 +979,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -996,8 +1003,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1495,7 +1500,70 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CF0E75F-879B-D04A-B404-34C072DAE15E}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>277</v>
+      </c>
+      <c r="B2">
+        <v>2025</v>
+      </c>
+      <c r="C2" t="s">
+        <v>276</v>
+      </c>
+      <c r="D2" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B3">
+        <v>2025</v>
+      </c>
+      <c r="C3" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>277</v>
+      </c>
+      <c r="B4">
+        <v>2025</v>
+      </c>
+      <c r="C4" t="s">
+        <v>287</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B7664C6-619C-FF44-887F-69948C30EFE6}">
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -1510,20 +1578,6 @@
       </c>
       <c r="D1" s="4" t="s">
         <v>275</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>277</v>
-      </c>
-      <c r="B2">
-        <v>2025</v>
-      </c>
-      <c r="C2" t="s">
-        <v>276</v>
-      </c>
-      <c r="D2" t="s">
-        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -1893,7 +1947,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F8CCDE5-1537-6F4F-8DCD-A875A6CFAFCD}">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="53.83203125" bestFit="1" customWidth="1"/>
@@ -1901,7 +1955,7 @@
     <col min="3" max="3" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>2</v>
       </c>
@@ -1918,25 +1972,24 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="13" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>284</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" t="s">
         <v>283</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" t="s">
         <v>285</v>
       </c>
-      <c r="F2" s="13"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -1953,7 +2006,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1970,7 +2023,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -1987,7 +2040,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -2004,7 +2057,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -2021,7 +2074,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>42</v>
       </c>
@@ -2038,7 +2091,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
@@ -2055,7 +2108,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>49</v>
       </c>
@@ -2072,7 +2125,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="7" t="s">
         <v>53</v>
       </c>
@@ -2089,7 +2142,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>56</v>
       </c>
@@ -2106,7 +2159,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>59</v>
       </c>
@@ -2123,7 +2176,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>62</v>
       </c>
@@ -2140,7 +2193,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>65</v>
       </c>
@@ -2157,7 +2210,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>67</v>
       </c>

</xml_diff>

<commit_message>
added last part of 2025 to cv
</commit_message>
<xml_diff>
--- a/data/CV_DA_2026.xlsx
+++ b/data/CV_DA_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10303"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/argyropoulos.d/Documents/GitHub/cv/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dionne/Documents/GitHub/cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7532620-2376-8944-8133-FD0196865BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4398C4-53E6-244A-BC6C-0252E15091FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="8" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
+    <workbookView xWindow="48960" yWindow="-1960" windowWidth="34200" windowHeight="20160" activeTab="11" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
   </bookViews>
   <sheets>
     <sheet name="positions" sheetId="11" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="668" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="377">
   <si>
     <t>degree</t>
   </si>
@@ -1173,6 +1173,12 @@
   </si>
   <si>
     <t>bioRxiv</t>
+  </si>
+  <si>
+    <t>Board</t>
+  </si>
+  <si>
+    <t>Sat as a coding expert on a board for hiring post-doctoral researchers at WEHI.</t>
   </si>
 </sst>
 </file>
@@ -1794,7 +1800,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C440642-50AF-EC46-A409-A4AFCC330B69}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -1842,6 +1848,17 @@
       </c>
       <c r="C4" t="s">
         <v>369</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B5">
+        <v>2025</v>
+      </c>
+      <c r="C5" t="s">
+        <v>376</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
make short version of cv
</commit_message>
<xml_diff>
--- a/data/CV_DA_2026.xlsx
+++ b/data/CV_DA_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10303"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dionne/Documents/GitHub/cv/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/argyropoulos.d/Documents/GitHub/cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4398C4-53E6-244A-BC6C-0252E15091FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737947FB-0D61-024F-8229-70389C84721A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48960" yWindow="-1960" windowWidth="34200" windowHeight="20160" activeTab="11" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
+    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
   </bookViews>
   <sheets>
     <sheet name="positions" sheetId="11" r:id="rId1"/>
@@ -23,8 +23,8 @@
     <sheet name="other_sci_comm" sheetId="8" r:id="rId8"/>
     <sheet name="publications" sheetId="9" r:id="rId9"/>
     <sheet name="tools" sheetId="12" r:id="rId10"/>
-    <sheet name="translational" sheetId="13" r:id="rId11"/>
-    <sheet name="other" sheetId="15" r:id="rId12"/>
+    <sheet name="other" sheetId="15" r:id="rId11"/>
+    <sheet name="translational" sheetId="13" r:id="rId12"/>
     <sheet name="training" sheetId="4" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="670" uniqueCount="377">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="399">
   <si>
     <t>degree</t>
   </si>
@@ -395,9 +395,6 @@
     <t>Malaria in Melbourne (MiM) Conference</t>
   </si>
   <si>
-    <t>2021</t>
-  </si>
-  <si>
     <t>Selected to attend Infection and Immunology conference in Lorne 2022.</t>
   </si>
   <si>
@@ -431,9 +428,6 @@
     <t>Stockholm International Youth Science Seminar Representative</t>
   </si>
   <si>
-    <t>Selected as the only Australian student a to represent the UoM. 25 countries selected one student to attend Nobel Prize Week events (including Ceremony and Banquet) and speak about their research. \href{https://ungaforskare.se/siyss/}{\faExternalLink}</t>
-  </si>
-  <si>
     <t>Communication for Research Scientists Three Minute Thesis (3MT) Runner-Up</t>
   </si>
   <si>
@@ -857,12 +851,6 @@
     <t>wastewateR</t>
   </si>
   <si>
-    <t>SeroTrackR R package provides the backbone for the PvSeroApp Shiny web application, with data processing of the multi-antigen serological data and applies the machine learning classification algorithm to identify individuals with recent exposure to P. vivax.  \href{https://github.com/dionnecargy/SeroTrackR/} {\faExternalLink} "GitHub"</t>
-  </si>
-  <si>
-    <t>The PvSeroApp Shiny web application streamlines the data processing of the multi-antigen Luminex-based Plasmodium vivax serological data and applies the machine learning classification algorithm to identify individuals with recent exposure to P. vivax.  \href{https://github.com/dionnecargy/PvSeroApp/} {\faExternalLink} "GitHub"</t>
-  </si>
-  <si>
     <t xml:space="preserve">ZiP Diagnostics </t>
   </si>
   <si>
@@ -911,18 +899,9 @@
     <t>Evaluating the Performance of Predicting Plasmodium vivax Infection Risk Using Serological Markers in Patients with Plasmodium falciparum Malaria</t>
   </si>
   <si>
-    <t xml:space="preserve">Tiedje, K. E., Zhan, Q., Ruybal-Pésantez, S., Tonkin-Hill, G., He, Q., Tan, M. H., Argyropoulos, D. C., Deed, S. L., Ghansah, A., Bangre, O., Oduro, A. R., Koram, K. A., Pascual, M. &amp; Day, K. P.  \href{https://doi.org/10.7554/eLife.91411.4} {\faExternalLink} "DOI" </t>
-  </si>
-  <si>
     <t>melbourne</t>
   </si>
   <si>
-    <t>wastewateR R package contains helper functions relevant for wasetwater-specific qPCR projects for in-house and collaborator needs.  \href{https://github.com/dionnecargy/wastewateR/} {\faExternalLink} "GitHub"</t>
-  </si>
-  <si>
-    <t>Developed melbourne R package with colour palette of melbourne tram network. \href{https://github.com/dionnecargy/melbourne/} {\faExternalLink} "GitHub"</t>
-  </si>
-  <si>
     <t>Women in Malaria 2025 Prize for Free Registration in 2026</t>
   </si>
   <si>
@@ -1040,12 +1019,6 @@
     <t xml:space="preserve">Won a raffle to have free attendance for the 2026 conference. </t>
   </si>
   <si>
-    <t xml:space="preserve">Awarded A\$1,500 to attend the European Summer Program in Infectious Disease Analysis and Modelling (ESPIDAM). </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Awarded A\$2,00 to attend the European Summer Program in Infectious Disease Analysis and Modelling (ESPIDAM).  \href{https://acreme.edu.au/ai-antibodies-and-equations-lessons-from-espidam-with-dionne-argyropoulos/}{\faExternalLink} "Write-up here" </t>
-  </si>
-  <si>
     <t xml:space="preserve">ACREME MASTER-MAP Travel and Training Award </t>
   </si>
   <si>
@@ -1118,33 +1091,9 @@
     <t xml:space="preserve">Organised by the ACREME committee, day focussed on mosquito vector-borne diseases. </t>
   </si>
   <si>
-    <t>Performance of SNP barcodes to determine genetic diversity and population structure of Plasmodium falciparum in Africa \href{https://doi.org/10.7554/eLife.91411.4} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Argyropoulos, D. C., Tan, M. H., Adobor, C., Mensah, B., Labbé, F., Tiedje, K. E., Koram, K. A., Ghansah, A. &amp; Day, K. P. \href{https://doi.org/ } {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Ghansah, A., Tiedje, K. E., Argyropoulos, D. C., Onwona, C. O., Deed, S. L., Labbé, F., Oduro, A. R., Koram, K. A., Pascual, M. &amp; Day, K. P. \href{https://doi.org/10.3389/fgene.2023.1071896} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Labbé, F., He, Q., Zhan, Q., Tiedje, K. E., Argyropoulos, D. C., Tan, M. H., Ghansah, A., Day, K. P. &amp; Pascual, M.\href{https://doi.org/10.3389/fpara.2023.1067966} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Tiedje, K.E., Oduro, A.R., Bangre, O., Amenga-Etego, L., Dadzie, S.K., Appawu, M.A., Frempong, K., Asoala, V., Ruybal-Pésantez, S., Narh, C.A., Deed, S.L., Argyropoulos, D. C., Ghansah, A., Agyei, S.A., Segbaya, S., Desewu, K., Williams, I., Simpson, J.A., Malm, K., Pascual, M., Koram, K.A. &amp; Day, K.P. \href{https://doi.org/10.1371/journal.pcbi.1010816} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Argyropoulos, D. C., Ruybal-Pesántez, S., Deed, S.L., Oduro, A.R., Dadzie, S.K., Appawu, M.A., Asoala, V., Pascual, M., Koram, K.A., Day, K.P. &amp; Tiedje, K.E. \href{https://doi.org/10.1371/journal.pgph.0000285} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
     <t>Hafidzah, M., Degaga, T. S., Christian, M., Alam, M. S., Hossain, M. S., Baird, J. K., Sutano, I., Smith, L., Argyropoulos, D., Amelia, A. R., Noviyanti, R., Price, R. N., Mueller, I., Thriemer, K. &amp; Longley, R. J.</t>
   </si>
   <si>
-    <t>Rios-Teran, C. A., Tiedje, K. E., Bangre, O., Deed, S. L., Argyropoulos, D. C., Koram, K. A., Oduro, A. R., Ansah, P. O. &amp; Day, K. P; \href{https://doi.org/10.1101/2025.08.15.25333797} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
-    <t>Bareng, P., Wu, K. W., Takashima, E., Argyropoulos, D., Smith, L., Naung, M., Mazhari, R., Schoffer, K., Kiernan-Walker, N., Abraham, A., Lamont, M., Mehra, S., Lim, P., Sattabongkot, J., Monteiro, W., Lacerda, M., Healer, J., Chitnis, C. E., Tham, W.-H., Tsuboi, T., Mueller, I., Barry, A. E. &amp; Longley, R. J.  \href{https://doi.org/10.1101/2025.07.07.663616} {\faExternalLink} "DOI"</t>
-  </si>
-  <si>
     <t>who</t>
   </si>
   <si>
@@ -1169,9 +1118,6 @@
     <t>Walter &amp; Eliza Hall Institute of Medical Research (WEHI)</t>
   </si>
   <si>
-    <t>medRxiv</t>
-  </si>
-  <si>
     <t>bioRxiv</t>
   </si>
   <si>
@@ -1179,6 +1125,126 @@
   </si>
   <si>
     <t>Sat as a coding expert on a board for hiring post-doctoral researchers at WEHI.</t>
+  </si>
+  <si>
+    <t>R/Medicine</t>
+  </si>
+  <si>
+    <t>posit::conf(2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conference to discuss R based tools and approaches in Medicine and Health Sciences. \href{https://rconsortium.github.io/RMedicine_website/}{\faExternalLink}. </t>
+  </si>
+  <si>
+    <t>Houston, US</t>
+  </si>
+  <si>
+    <t>Conference to discuss latest developments in R and Python. \href{https://conf.posit.co/2026/}{\faExternalLink}.</t>
+  </si>
+  <si>
+    <t>Scholarship</t>
+  </si>
+  <si>
+    <t>Posit PBC</t>
+  </si>
+  <si>
+    <t>Opportunity Scholar for posit::conf(2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The PvSeroApp Shiny web application streamlines the data processing of the multi-antigen Luminex-based Plasmodium vivax serological data and applies the machine learning classification algorithm to identify individuals with recent exposure to P. vivax.  \href{https://github.com/dionnecargy/PvSeroApp/} {\faExternalLink} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SeroTrackR R package provides the backbone for the PvSeroApp Shiny web application, with data processing of the multi-antigen serological data and applies the machine learning classification algorithm to identify individuals with recent exposure to P. vivax.  \href{https://github.com/dionnecargy/SeroTrackR/} {\faExternalLink} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">wastewateR R package contains helper functions relevant for wasetwater-specific qPCR projects for in-house and collaborator needs.  \href{https://github.com/dionnecargy/wastewateR/} {\faExternalLink} </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Developed melbourne R package with colour palette of melbourne tram network. \href{https://github.com/dionnecargy/melbourne/} {\faExternalLink} </t>
+  </si>
+  <si>
+    <t>doi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rios-Teran, C. A., Tiedje, K. E., Bangre, O., Deed, S. L., Argyropoulos, D. C., Koram, K. A., Oduro, A. R., Ansah, P. O. &amp; Day, K. P </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bareng, P., Wu, K. W., Takashima, E., Argyropoulos, D., Smith, L., Naung, M., Mazhari, R., Schoffer, K., Kiernan-Walker, N., Abraham, A., Lamont, M., Mehra, S., Lim, P., Sattabongkot, J., Monteiro, W., Lacerda, M., Healer, J., Chitnis, C. E., Tham, W.-H., Tsuboi, T., Mueller, I., Barry, A. E. &amp; Longley, R. J. </t>
+  </si>
+  <si>
+    <t>Tiedje, K. E., Zhan, Q., Ruybal-Pésantez, S., Tonkin-Hill, G., He, Q., Tan, M. H., Argyropoulos, D. C., Deed, S. L., Ghansah, A., Bangre, O., Oduro, A. R., Koram, K. A., Pascual, M. &amp; Day, K. P.</t>
+  </si>
+  <si>
+    <t>Argyropoulos, D. C., Tan, M. H., Adobor, C., Mensah, B., Labbé, F., Tiedje, K. E., Koram, K. A., Ghansah, A. &amp; Day, K. P.</t>
+  </si>
+  <si>
+    <t>Ghansah, A., Tiedje, K. E., Argyropoulos, D. C., Onwona, C. O., Deed, S. L., Labbé, F., Oduro, A. R., Koram, K. A., Pascual, M. &amp; Day, K. P.</t>
+  </si>
+  <si>
+    <t>Labbé, F., He, Q., Zhan, Q., Tiedje, K. E., Argyropoulos, D. C., Tan, M. H., Ghansah, A., Day, K. P. &amp; Pascual, M.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tiedje, K.E., Oduro, A.R., Bangre, O., Amenga-Etego, L., Dadzie, S.K., Appawu, M.A., Frempong, K., Asoala, V., Ruybal-Pésantez, S., Narh, C.A., Deed, S.L., Argyropoulos, D. C., Ghansah, A., Agyei, S.A., Segbaya, S., Desewu, K., Williams, I., Simpson, J.A., Malm, K., Pascual, M., Koram, K.A. &amp; Day, K.P. </t>
+  </si>
+  <si>
+    <t>Argyropoulos, D. C., Ruybal-Pesántez, S., Deed, S.L., Oduro, A.R., Dadzie, S.K., Appawu, M.A., Asoala, V., Pascual, M., Koram, K.A., Day, K.P. &amp; Tiedje, K.E.</t>
+  </si>
+  <si>
+    <t>Journal of Infectious Diseases</t>
+  </si>
+  <si>
+    <t>PLoS Neglected Tropical Diseases</t>
+  </si>
+  <si>
+    <t>Performance of SNP barcodes to determine genetic diversity and population structure of Plasmodium falciparum in Africa</t>
+  </si>
+  <si>
+    <t>doi.org/1371/journal.pntd.0014174</t>
+  </si>
+  <si>
+    <t>doi.org/1101/2025.08.15.25333797</t>
+  </si>
+  <si>
+    <t>doi.org/1093/infdis/jiag164</t>
+  </si>
+  <si>
+    <t>doi.org/7554/eLife.91411.4</t>
+  </si>
+  <si>
+    <t>doi.org/3389/fgene.2023.1071896</t>
+  </si>
+  <si>
+    <t>doi.org/3389/fpara.2023.1067966</t>
+  </si>
+  <si>
+    <t>doi.org/1371/journal.pcbi.1010816</t>
+  </si>
+  <si>
+    <t>doi.org/1371/journal.pgph.0000285</t>
+  </si>
+  <si>
+    <t>doi.org/1111/mec.16029</t>
+  </si>
+  <si>
+    <t>selected</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>Awarded A\$1,500 to attend the European Summer Program in Infectious Disease Analysis and Modelling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Awarded A\$2,00 to attend the European Summer Program in Infectious Disease Analysis and Modelling.  \href{https://acreme.edu.au/ai-antibodies-and-equations-lessons-from-espidam-with-dionne-argyropoulos/}{\faExternalLink} "Write-up here" </t>
+  </si>
+  <si>
+    <t>Awarded full scholarship to attend the posit::conf(2026) inclusive of travel, incidentals, hotel, conference and workshop registration \href{https://conf.posit.co/2026/}{\faExternalLink}.</t>
+  </si>
+  <si>
+    <t>Selected as the only Australian student a to represent the UoM. 25 countries selected one student to attend Nobel Prize Week events. \href{https://ungaforskare.se/siyss/}{\faExternalLink}</t>
   </si>
 </sst>
 </file>
@@ -1657,19 +1723,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B2" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="C2" t="s">
-        <v>372</v>
+        <v>355</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -1687,72 +1753,72 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B2">
         <v>2025</v>
       </c>
       <c r="C2" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D2" t="s">
-        <v>270</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B3">
         <v>2025</v>
       </c>
       <c r="C3" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D3" t="s">
-        <v>269</v>
+        <v>368</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B4">
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D4" t="s">
-        <v>289</v>
+        <v>369</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B5">
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="D5" t="s">
-        <v>290</v>
+        <v>370</v>
       </c>
     </row>
   </sheetData>
@@ -1761,104 +1827,104 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C440642-50AF-EC46-A409-A4AFCC330B69}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="D1" s="13" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2">
+        <v>2025</v>
+      </c>
+      <c r="C2" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="B3">
+        <v>2025</v>
+      </c>
+      <c r="C3" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B4">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="12" t="s">
+        <v>357</v>
+      </c>
+      <c r="B5">
+        <v>2025</v>
+      </c>
+      <c r="C5" t="s">
+        <v>358</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B7664C6-619C-FF44-887F-69948C30EFE6}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>258</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B2">
         <v>2025</v>
       </c>
       <c r="C2" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="D2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C440642-50AF-EC46-A409-A4AFCC330B69}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="13" t="s">
-        <v>134</v>
-      </c>
-      <c r="B1" s="13" t="s">
-        <v>258</v>
-      </c>
-      <c r="C1" s="13" t="s">
-        <v>260</v>
-      </c>
-      <c r="D1" s="13" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="12" t="s">
-        <v>297</v>
-      </c>
-      <c r="B2">
-        <v>2025</v>
-      </c>
-      <c r="C2" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="12" t="s">
-        <v>297</v>
-      </c>
-      <c r="B3">
-        <v>2025</v>
-      </c>
-      <c r="C3" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="12" t="s">
-        <v>298</v>
-      </c>
-      <c r="B4">
-        <v>2026</v>
-      </c>
-      <c r="C4" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="12" t="s">
-        <v>375</v>
-      </c>
-      <c r="B5">
-        <v>2025</v>
-      </c>
-      <c r="C5" t="s">
-        <v>376</v>
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -1893,13 +1959,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="D2" s="19">
         <v>2025</v>
@@ -1907,13 +1973,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>334</v>
+        <v>325</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="D3" s="19">
         <v>2025</v>
@@ -1921,10 +1987,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
@@ -1935,10 +2001,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
@@ -1949,10 +2015,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B6" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C6" t="s">
         <v>8</v>
@@ -1963,10 +2029,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B7" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
@@ -2510,217 +2576,217 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>366</v>
+        <v>349</v>
       </c>
       <c r="B2" s="17">
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>367</v>
+        <v>350</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11" t="s">
-        <v>368</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B3" s="17">
         <v>2026</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="11" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B4" s="17">
         <v>2026</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="11" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B5" s="18">
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="E5" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B6" s="17">
         <v>2025</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="11" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B7" s="17">
         <v>2025</v>
       </c>
       <c r="C7" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B8" s="6">
         <v>2023</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B9" s="6">
         <v>2022</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B12" s="18">
         <v>2021</v>
       </c>
       <c r="C12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E12" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B13" s="18">
         <v>2021</v>
       </c>
       <c r="C13" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E13" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B14" s="18" t="s">
         <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E14" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B15" s="18">
         <v>2019</v>
       </c>
       <c r="C15" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E15" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B16" s="18">
         <v>2019</v>
       </c>
       <c r="C16" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E16" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.2">
@@ -2800,159 +2866,188 @@
       <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13"/>
+      <c r="F1" s="13" t="s">
+        <v>392</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>315</v>
+        <v>308</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="E3" t="s">
-        <v>306</v>
+        <v>299</v>
+      </c>
+      <c r="F3" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="E4" t="s">
-        <v>310</v>
+        <v>303</v>
+      </c>
+      <c r="F4" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="E5" t="s">
-        <v>311</v>
+        <v>304</v>
+      </c>
+      <c r="F5" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>319</v>
+        <v>312</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="E7" t="s">
-        <v>321</v>
+        <v>314</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="E8" t="s">
-        <v>324</v>
+        <v>317</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>328</v>
+        <v>321</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C10" t="s">
         <v>45</v>
       </c>
       <c r="D10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="E10" t="s">
-        <v>302</v>
+        <v>295</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -2960,7 +3055,7 @@
         <v>25</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C11" t="s">
         <v>26</v>
@@ -2969,7 +3064,10 @@
         <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>307</v>
+        <v>300</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>393</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -2977,7 +3075,7 @@
         <v>28</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="C12" t="s">
         <v>29</v>
@@ -2987,6 +3085,9 @@
       </c>
       <c r="E12" t="s">
         <v>30</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -3005,6 +3106,9 @@
       <c r="E13" t="s">
         <v>33</v>
       </c>
+      <c r="F13" s="11" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -3022,6 +3126,9 @@
       <c r="E14" t="s">
         <v>36</v>
       </c>
+      <c r="F14" s="11" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -3039,6 +3146,9 @@
       <c r="E15" t="s">
         <v>39</v>
       </c>
+      <c r="F15" s="11" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -3051,13 +3161,16 @@
         <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="E16" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="7" t="s">
         <v>43</v>
       </c>
@@ -3068,13 +3181,16 @@
         <v>45</v>
       </c>
       <c r="D17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E17" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -3090,8 +3206,11 @@
       <c r="E18" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="s">
         <v>51</v>
       </c>
@@ -3107,8 +3226,11 @@
       <c r="E19" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -3124,8 +3246,11 @@
       <c r="E20" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -3141,8 +3266,11 @@
       <c r="E21" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -3158,8 +3286,11 @@
       <c r="E22" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>63</v>
       </c>
@@ -3175,8 +3306,11 @@
       <c r="E23" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -3192,8 +3326,11 @@
       <c r="E24" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -3209,8 +3346,11 @@
       <c r="E25" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>70</v>
       </c>
@@ -3226,8 +3366,11 @@
       <c r="E26" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="7" t="s">
         <v>72</v>
       </c>
@@ -3243,8 +3386,11 @@
       <c r="E27" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="7" t="s">
         <v>75</v>
       </c>
@@ -3260,8 +3406,11 @@
       <c r="E28" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="7" t="s">
         <v>78</v>
       </c>
@@ -3277,14 +3426,17 @@
       <c r="E29" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F29" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B30"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B31"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B32"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.2">
@@ -3345,50 +3497,50 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -3401,7 +3553,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADD646AB-7E33-9A4A-B118-8FB38A78DA5A}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="64.83203125" bestFit="1" customWidth="1"/>
@@ -3409,7 +3561,7 @@
     <col min="3" max="3" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="11" t="s">
         <v>108</v>
       </c>
@@ -3420,233 +3572,298 @@
         <v>1</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B2" t="s">
-        <v>293</v>
+      <c r="F1" s="11" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>366</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>365</v>
       </c>
       <c r="C2" s="11">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D2" s="14">
-        <v>45735</v>
-      </c>
-      <c r="E2" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+        <v>46128</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>397</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>333</v>
+        <v>284</v>
       </c>
       <c r="B3" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="C3" s="11">
         <v>2025</v>
       </c>
       <c r="D3" s="14">
-        <v>45795</v>
+        <v>45735</v>
       </c>
       <c r="E3" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>322</v>
+      </c>
+      <c r="F3" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>332</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>309</v>
+        <v>324</v>
+      </c>
+      <c r="B4" t="s">
+        <v>287</v>
       </c>
       <c r="C4" s="11">
         <v>2025</v>
       </c>
       <c r="D4" s="14">
+        <v>45795</v>
+      </c>
+      <c r="E4" t="s">
+        <v>395</v>
+      </c>
+      <c r="F4" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>323</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="C5" s="11">
+        <v>2025</v>
+      </c>
+      <c r="D5" s="14">
         <v>45789</v>
       </c>
-      <c r="E4" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="11" t="s">
+      <c r="E5" t="s">
+        <v>396</v>
+      </c>
+      <c r="F5" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>111</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C6" s="15" t="s">
-        <v>32</v>
+      <c r="C6" s="11">
+        <v>2024</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>115</v>
+        <v>87</v>
+      </c>
+      <c r="C7" s="11">
+        <v>2024</v>
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="11" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+        <v>112</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="15" t="s">
-        <v>48</v>
+        <v>114</v>
+      </c>
+      <c r="C8" s="11">
+        <v>2021</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+        <v>115</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C9" s="15" t="s">
-        <v>48</v>
+        <v>117</v>
+      </c>
+      <c r="C9" s="11">
+        <v>2019</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>118</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>48</v>
+        <v>117</v>
+      </c>
+      <c r="C10" s="11">
+        <v>2019</v>
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B11" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>48</v>
+      <c r="C11" s="11">
+        <v>2019</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>48</v>
+      <c r="C12" s="11">
+        <v>2019</v>
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="15" t="s">
-        <v>48</v>
+      <c r="C13" s="11">
+        <v>2019</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+        <v>398</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C14" s="15" t="s">
-        <v>76</v>
+      <c r="C14" s="11">
+        <v>2019</v>
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+        <v>127</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>76</v>
+        <v>87</v>
+      </c>
+      <c r="C15" s="11">
+        <v>2018</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="C16" s="6"/>
+        <v>129</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C16" s="11">
+        <v>2018</v>
+      </c>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.2">
       <c r="C17" s="6"/>
+    </row>
+    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C18" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3655,7 +3872,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD52188-922E-CF44-BFD0-18928D31283D}">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" customWidth="1"/>
@@ -3663,18 +3880,18 @@
     <col min="6" max="6" width="20.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>24</v>
@@ -3685,625 +3902,765 @@
       <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>196</v>
+      <c r="H1" s="4" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>360</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>264</v>
+        <v>306</v>
       </c>
       <c r="C2" s="12">
+        <v>46279</v>
+      </c>
+      <c r="D2" s="12">
+        <v>46281</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>306</v>
+      </c>
+      <c r="C3" s="12">
+        <v>46147</v>
+      </c>
+      <c r="D3" s="12">
+        <v>46150</v>
+      </c>
+      <c r="E3" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C4" s="12">
         <v>45960</v>
       </c>
-      <c r="D2" s="12">
+      <c r="D4" s="12">
         <v>45961</v>
       </c>
-      <c r="E2" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B3" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="C3" s="12">
-        <v>45735</v>
-      </c>
-      <c r="D3" s="12">
-        <v>45736</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="F3" s="11" t="s">
-        <v>340</v>
-      </c>
-      <c r="G3" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>347</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="C4" s="12">
-        <v>45943</v>
-      </c>
-      <c r="D4" s="12">
-        <v>45944</v>
-      </c>
       <c r="E4" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G4" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+        <v>340</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>348</v>
+        <v>184</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C5" s="12">
+        <v>45735</v>
+      </c>
+      <c r="D5" s="12">
+        <v>45736</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>331</v>
+      </c>
+      <c r="G5" t="s">
+        <v>341</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>338</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C6" s="12">
+        <v>45943</v>
+      </c>
+      <c r="D6" s="12">
+        <v>45944</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>342</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>339</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" s="12">
         <v>45838</v>
       </c>
-      <c r="D5" s="12">
+      <c r="D7" s="12">
         <v>45841</v>
       </c>
-      <c r="E5" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="F5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>334</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="C6" s="12">
-        <v>45831</v>
-      </c>
-      <c r="D6" s="12">
-        <v>45835</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>183</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="G6" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>227</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="C7" s="12">
-        <v>45783</v>
-      </c>
-      <c r="D7" s="12">
-        <v>45783</v>
-      </c>
       <c r="E7" s="11" t="s">
-        <v>29</v>
+        <v>180</v>
       </c>
       <c r="F7" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" s="11" customFormat="1" x14ac:dyDescent="0.2">
+        <v>343</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>295</v>
+        <v>325</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="C8" s="12">
+        <v>45831</v>
+      </c>
+      <c r="D8" s="12">
+        <v>45835</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G8" t="s">
+        <v>344</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C9" s="12">
+        <v>45783</v>
+      </c>
+      <c r="D9" s="12">
+        <v>45783</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" t="s">
+        <v>345</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>288</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C10" s="12">
         <v>45889</v>
       </c>
-      <c r="D8" s="12">
+      <c r="D10" s="12">
         <v>45889</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="F8" s="11" t="s">
+      <c r="E10" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="F10" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G8" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="G10" t="s">
+        <v>346</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s">
+        <v>329</v>
+      </c>
+      <c r="F11" t="s">
         <v>213</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="G11" t="s">
+        <v>244</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>190</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E9" t="s">
-        <v>338</v>
-      </c>
-      <c r="F9" t="s">
-        <v>215</v>
-      </c>
-      <c r="G9" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="E12" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E10" t="s">
-        <v>183</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="G12" t="s">
+        <v>242</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>194</v>
       </c>
-      <c r="G10" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>196</v>
-      </c>
-      <c r="B11" s="6" t="s">
+      <c r="B13" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E11" t="s">
-        <v>183</v>
-      </c>
-      <c r="F11" t="s">
+      <c r="E13" t="s">
+        <v>181</v>
+      </c>
+      <c r="F13" t="s">
         <v>41</v>
       </c>
-      <c r="G11" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>214</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="G13" t="s">
+        <v>240</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>212</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E12" t="s">
-        <v>183</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="E14" t="s">
+        <v>181</v>
+      </c>
+      <c r="F14" t="s">
         <v>8</v>
       </c>
-      <c r="G12" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>230</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E13" t="s">
-        <v>29</v>
-      </c>
-      <c r="F13" t="s">
-        <v>190</v>
-      </c>
-      <c r="G13" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>188</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E14" t="s">
-        <v>29</v>
-      </c>
-      <c r="F14" t="s">
-        <v>190</v>
-      </c>
       <c r="G14" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+        <v>245</v>
+      </c>
+      <c r="H14" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>185</v>
-      </c>
-      <c r="B15" s="6">
-        <v>2021</v>
+        <v>228</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="E15" t="s">
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G15" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="6">
-        <v>2021</v>
+      <c r="B16" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="E16" t="s">
-        <v>182</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="G16" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+      <c r="H16" s="11" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="B17" s="6">
         <v>2021</v>
       </c>
       <c r="E17" t="s">
-        <v>182</v>
+        <v>29</v>
       </c>
       <c r="F17" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="G17" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+      <c r="H17" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="B18" s="6">
         <v>2021</v>
       </c>
       <c r="E18" t="s">
-        <v>338</v>
+        <v>180</v>
       </c>
       <c r="F18" t="s">
+        <v>191</v>
+      </c>
+      <c r="G18" t="s">
+        <v>243</v>
+      </c>
+      <c r="H18" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>193</v>
-      </c>
-      <c r="G18" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>198</v>
       </c>
       <c r="B19" s="6">
         <v>2021</v>
       </c>
       <c r="E19" t="s">
+        <v>180</v>
+      </c>
+      <c r="F19" t="s">
+        <v>191</v>
+      </c>
+      <c r="G19" t="s">
+        <v>239</v>
+      </c>
+      <c r="H19" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>194</v>
+      </c>
+      <c r="B20" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E20" t="s">
+        <v>329</v>
+      </c>
+      <c r="F20" t="s">
+        <v>191</v>
+      </c>
+      <c r="G20" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>196</v>
+      </c>
+      <c r="B21" s="6">
+        <v>2021</v>
+      </c>
+      <c r="E21" t="s">
         <v>29</v>
       </c>
-      <c r="F19" t="s">
-        <v>193</v>
-      </c>
-      <c r="G19" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>188</v>
-      </c>
-      <c r="B20" s="6">
-        <v>2020</v>
-      </c>
-      <c r="E20" t="s">
-        <v>182</v>
-      </c>
-      <c r="F20" t="s">
-        <v>189</v>
-      </c>
-      <c r="G20" t="s">
+      <c r="F21" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>192</v>
-      </c>
-      <c r="B21" s="6">
-        <v>2020</v>
-      </c>
-      <c r="E21" t="s">
-        <v>183</v>
-      </c>
-      <c r="F21" t="s">
-        <v>194</v>
-      </c>
       <c r="G21" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+        <v>209</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>240</v>
+        <v>186</v>
       </c>
       <c r="B22" s="6">
         <v>2020</v>
       </c>
       <c r="E22" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F22" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="G22" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+      <c r="H22" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B23" s="6">
         <v>2020</v>
       </c>
       <c r="E23" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F23" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G23" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+      <c r="H23" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="B24" s="6">
         <v>2020</v>
       </c>
       <c r="E24" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F24" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G24" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+      <c r="H24" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>196</v>
       </c>
       <c r="B25" s="6">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E25" t="s">
-        <v>338</v>
+        <v>180</v>
       </c>
       <c r="F25" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="G25" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>232</v>
+      </c>
+      <c r="H25" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B26" s="6">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E26" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F26" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="G26" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+        <v>236</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B27" s="6">
         <v>2019</v>
       </c>
       <c r="E27" t="s">
-        <v>209</v>
+        <v>329</v>
       </c>
       <c r="F27" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="G27" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+      <c r="H27" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B28" s="6">
         <v>2019</v>
       </c>
       <c r="E28" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F28" t="s">
+        <v>195</v>
+      </c>
+      <c r="G28" t="s">
+        <v>233</v>
+      </c>
+      <c r="H28" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" s="6">
+        <v>2019</v>
+      </c>
+      <c r="E29" t="s">
+        <v>207</v>
+      </c>
+      <c r="F29" t="s">
+        <v>202</v>
+      </c>
+      <c r="G29" t="s">
         <v>206</v>
       </c>
-      <c r="G28" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>199</v>
-      </c>
-      <c r="B29" s="6">
-        <v>2018</v>
-      </c>
-      <c r="E29" t="s">
-        <v>182</v>
-      </c>
-      <c r="F29" t="s">
-        <v>206</v>
-      </c>
-      <c r="G29" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H29" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>201</v>
       </c>
       <c r="B30" s="6">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E30" t="s">
-        <v>339</v>
+        <v>181</v>
       </c>
       <c r="F30" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G30" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+      <c r="H30" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B31" s="6">
         <v>2018</v>
       </c>
       <c r="E31" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F31" t="s">
-        <v>8</v>
+        <v>204</v>
       </c>
       <c r="G31" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+        <v>237</v>
+      </c>
+      <c r="H31" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B32" s="6">
         <v>2018</v>
       </c>
       <c r="E32" t="s">
-        <v>182</v>
+        <v>330</v>
       </c>
       <c r="F32" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="G32" t="s">
+        <v>208</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>200</v>
+      </c>
+      <c r="B33" s="6">
+        <v>2018</v>
+      </c>
+      <c r="E33" t="s">
+        <v>180</v>
+      </c>
+      <c r="F33" t="s">
+        <v>8</v>
+      </c>
+      <c r="G33" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="36" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E36" s="6"/>
-      <c r="F36" s="6"/>
-    </row>
-    <row r="37" spans="5:6" x14ac:dyDescent="0.2">
-      <c r="E37" s="6"/>
-      <c r="F37" s="6"/>
-    </row>
-    <row r="38" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="H33" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>201</v>
+      </c>
+      <c r="B34" s="6">
+        <v>2018</v>
+      </c>
+      <c r="E34" t="s">
+        <v>180</v>
+      </c>
+      <c r="F34" t="s">
+        <v>205</v>
+      </c>
+      <c r="G34" t="s">
+        <v>234</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
     </row>
-    <row r="39" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
     </row>
-    <row r="40" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
     </row>
-    <row r="41" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
     </row>
-    <row r="42" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
     </row>
-    <row r="43" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E43" s="6"/>
       <c r="F43" s="6"/>
     </row>
-    <row r="44" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
     </row>
-    <row r="45" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E45" s="6"/>
       <c r="F45" s="6"/>
     </row>
-    <row r="46" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E46" s="6"/>
       <c r="F46" s="6"/>
     </row>
-    <row r="47" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E47" s="6"/>
       <c r="F47" s="6"/>
     </row>
-    <row r="48" spans="5:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E48" s="6"/>
       <c r="F48" s="6"/>
     </row>
@@ -4327,9 +4684,17 @@
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
     </row>
+    <row r="54" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+    </row>
+    <row r="55" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E55" s="6"/>
+      <c r="F55" s="6"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:G32">
-    <sortCondition descending="1" ref="B1:B32"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A17:G34">
+    <sortCondition descending="1" ref="B1:B34"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4353,7 +4718,7 @@
         <v>23</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>3</v>
@@ -4364,87 +4729,87 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="B2" s="11">
         <v>2025</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>343</v>
+        <v>334</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B3">
         <v>2024</v>
       </c>
       <c r="C3" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" t="s">
         <v>136</v>
-      </c>
-      <c r="D3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E3" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B4">
         <v>2022</v>
       </c>
       <c r="C4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B5">
         <v>2021</v>
       </c>
       <c r="C5" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D5" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B6">
         <v>2021</v>
       </c>
       <c r="C6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -4455,13 +4820,13 @@
         <v>2019</v>
       </c>
       <c r="C7" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D7" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E7" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -4472,13 +4837,13 @@
         <v>2019</v>
       </c>
       <c r="C8" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -4489,13 +4854,13 @@
         <v>2018</v>
       </c>
       <c r="C9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -4506,13 +4871,13 @@
         <v>2018</v>
       </c>
       <c r="C10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -4525,152 +4890,212 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48A8CE42-696C-CE44-B442-78C1AB999450}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28.1640625" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
     <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="61.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+      <c r="E1" s="13" t="s">
+        <v>371</v>
+      </c>
+      <c r="F1" s="13" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="B2" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C2">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D2" t="s">
-        <v>363</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+        <v>372</v>
+      </c>
+      <c r="E2" t="s">
+        <v>383</v>
+      </c>
+      <c r="F2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="B3" t="s">
-        <v>374</v>
+        <v>356</v>
       </c>
       <c r="C3">
         <v>2025</v>
       </c>
       <c r="D3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+        <v>373</v>
+      </c>
+      <c r="E3" t="s">
+        <v>384</v>
+      </c>
+      <c r="F3" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="B4" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="C4">
         <v>2025</v>
       </c>
       <c r="D4" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+      <c r="E4" t="s">
+        <v>385</v>
+      </c>
+      <c r="F4" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C5">
         <v>2025</v>
       </c>
       <c r="D5" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+        <v>374</v>
+      </c>
+      <c r="E5" t="s">
+        <v>386</v>
+      </c>
+      <c r="F5" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>356</v>
+        <v>382</v>
       </c>
       <c r="B6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C6">
         <v>2023</v>
       </c>
       <c r="D6" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+        <v>375</v>
+      </c>
+      <c r="E6" t="s">
+        <v>387</v>
+      </c>
+      <c r="F6" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B7" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C7">
         <v>2023</v>
       </c>
       <c r="D7" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+        <v>376</v>
+      </c>
+      <c r="E7" t="s">
+        <v>388</v>
+      </c>
+      <c r="F7" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C8">
         <v>2023</v>
       </c>
       <c r="D8" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+        <v>377</v>
+      </c>
+      <c r="E8" t="s">
+        <v>389</v>
+      </c>
+      <c r="F8" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C9">
         <v>2022</v>
       </c>
       <c r="D9" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+        <v>378</v>
+      </c>
+      <c r="E9" t="s">
+        <v>390</v>
+      </c>
+      <c r="F9" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B10" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C10">
         <v>2021</v>
       </c>
       <c r="D10" t="s">
-        <v>361</v>
+        <v>379</v>
+      </c>
+      <c r="E10" t="s">
+        <v>391</v>
+      </c>
+      <c r="F10" t="s">
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated as of sept 2026
</commit_message>
<xml_diff>
--- a/data/CV_DA_2026.xlsx
+++ b/data/CV_DA_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10901"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/argyropoulos.d/Documents/GitHub/cv/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dionne/Documents/GitHub/cv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{737947FB-0D61-024F-8229-70389C84721A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67ABB5B-5AF2-A749-80C6-7A136B42CDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="5" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
+    <workbookView xWindow="58760" yWindow="-2420" windowWidth="34200" windowHeight="20140" activeTab="8" xr2:uid="{2F9E9AA9-9FED-064E-A335-70CF639738A5}"/>
   </bookViews>
   <sheets>
     <sheet name="positions" sheetId="11" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="407">
   <si>
     <t>degree</t>
   </si>
@@ -878,12 +878,6 @@
     <t>Tutor for Introduction to R Course, WEHI</t>
   </si>
   <si>
-    <t>Workshop Developer, Tutor, Demonstrator for BIOL90042</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aided development of machine learning workshop and proof-read other workshop materials for R-based coding subject. Taught machine learning workshop. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Delivered ggplot2 plotting tutorial and assisted in tutoring WEHI students and staff in R coding. </t>
   </si>
   <si>
@@ -1118,9 +1112,6 @@
     <t>Walter &amp; Eliza Hall Institute of Medical Research (WEHI)</t>
   </si>
   <si>
-    <t>bioRxiv</t>
-  </si>
-  <si>
     <t>Board</t>
   </si>
   <si>
@@ -1202,9 +1193,6 @@
     <t>doi.org/1371/journal.pntd.0014174</t>
   </si>
   <si>
-    <t>doi.org/1101/2025.08.15.25333797</t>
-  </si>
-  <si>
     <t>doi.org/1093/infdis/jiag164</t>
   </si>
   <si>
@@ -1245,6 +1233,42 @@
   </si>
   <si>
     <t>Selected as the only Australian student a to represent the UoM. 25 countries selected one student to attend Nobel Prize Week events. \href{https://ungaforskare.se/siyss/}{\faExternalLink}</t>
+  </si>
+  <si>
+    <t>Workshop Developer, Head Tutor for BIOL90042: "Coding and Data Analysis in Biomedicine"</t>
+  </si>
+  <si>
+    <t>Climate Sensitive Infectious Diseases Network Regional Meeting</t>
+  </si>
+  <si>
+    <t>Kanchanaburi, Thailand</t>
+  </si>
+  <si>
+    <t>Inaugural regional meeting for CSIDNet in Asia-Pacific. 15-minute talk. Part of SPARLE Team and aided R-based tutorial on infectious disease epidemiological modelling.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">doi.org/10.1016/j.lanmic.2025.101335 </t>
+  </si>
+  <si>
+    <t>The Lancet Microbe</t>
+  </si>
+  <si>
+    <t>Development of workshop and tutorial materials; R-based coding subject. Taught Epidemiology and ML workshops.</t>
+  </si>
+  <si>
+    <t>Computer Sciences Initiative Seminar</t>
+  </si>
+  <si>
+    <t>Best Speaker at the Computer Sciences Initiative Seminar</t>
+  </si>
+  <si>
+    <t>Doherty Institute</t>
+  </si>
+  <si>
+    <t>Conference inviting all Parkville Precinct members researching ID modelling</t>
+  </si>
+  <si>
+    <t>Awarded A\$500 Prize for Best Talk</t>
   </si>
 </sst>
 </file>
@@ -1729,7 +1753,7 @@
         <v>270</v>
       </c>
       <c r="C2" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="D2" t="s">
         <v>8</v>
@@ -1776,7 +1800,7 @@
         <v>259</v>
       </c>
       <c r="D2" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -1790,7 +1814,7 @@
         <v>265</v>
       </c>
       <c r="D3" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -1804,7 +1828,7 @@
         <v>266</v>
       </c>
       <c r="D4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -1815,10 +1839,10 @@
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -1842,51 +1866,51 @@
         <v>258</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B2">
         <v>2025</v>
       </c>
       <c r="C2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B3">
         <v>2025</v>
       </c>
       <c r="C3" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B4">
         <v>2026</v>
       </c>
       <c r="C4" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="12" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="B5">
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
   </sheetData>
@@ -1959,13 +1983,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D2" s="19">
         <v>2025</v>
@@ -1973,13 +1997,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="D3" s="19">
         <v>2025</v>
@@ -2551,7 +2575,7 @@
   <cols>
     <col min="1" max="1" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.83203125" style="18" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="75.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="255.83203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.1640625" customWidth="1"/>
@@ -2576,17 +2600,17 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="B2" s="17">
         <v>2026</v>
       </c>
       <c r="C2" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D2" s="11"/>
       <c r="E2" s="11" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -2597,11 +2621,11 @@
         <v>2026</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>276</v>
+        <v>395</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="11" t="s">
-        <v>277</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -2616,7 +2640,7 @@
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="11" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -2627,10 +2651,10 @@
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="E5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -2645,7 +2669,7 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -2656,11 +2680,11 @@
         <v>2025</v>
       </c>
       <c r="C7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="D7" s="4"/>
       <c r="E7" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -2867,112 +2891,112 @@
         <v>4</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="C2" s="11" t="s">
         <v>305</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="D2" s="11" t="s">
+        <v>303</v>
+      </c>
+      <c r="E2" s="11" t="s">
         <v>306</v>
       </c>
-      <c r="C2" s="11" t="s">
-        <v>307</v>
-      </c>
-      <c r="D2" s="11" t="s">
-        <v>305</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>308</v>
-      </c>
       <c r="F2" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="B3" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D3" s="11" t="s">
+        <v>295</v>
+      </c>
+      <c r="E3" t="s">
         <v>297</v>
       </c>
-      <c r="E3" t="s">
-        <v>299</v>
-      </c>
       <c r="F3" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B4" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C4" s="11" t="s">
+        <v>299</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="E4" t="s">
         <v>301</v>
       </c>
-      <c r="D4" s="11" t="s">
-        <v>302</v>
-      </c>
-      <c r="E4" t="s">
-        <v>303</v>
-      </c>
       <c r="F4" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="B5" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="D5" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="E5" t="s">
         <v>302</v>
       </c>
-      <c r="E5" t="s">
-        <v>304</v>
-      </c>
       <c r="F5" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="11" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>262</v>
@@ -2981,53 +3005,53 @@
         <v>29</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="E7" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D8" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="E8" t="s">
         <v>315</v>
       </c>
-      <c r="E8" t="s">
-        <v>317</v>
-      </c>
       <c r="F8" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C9" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>316</v>
+      </c>
+      <c r="E9" s="11" t="s">
         <v>319</v>
       </c>
-      <c r="D9" s="11" t="s">
-        <v>318</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>321</v>
-      </c>
       <c r="F9" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -3044,10 +3068,10 @@
         <v>263</v>
       </c>
       <c r="E10" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -3064,10 +3088,10 @@
         <v>27</v>
       </c>
       <c r="E11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -3075,7 +3099,7 @@
         <v>28</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C12" t="s">
         <v>29</v>
@@ -3087,7 +3111,7 @@
         <v>30</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
@@ -3107,7 +3131,7 @@
         <v>33</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -3127,7 +3151,7 @@
         <v>36</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
@@ -3147,7 +3171,7 @@
         <v>39</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
@@ -3161,13 +3185,13 @@
         <v>38</v>
       </c>
       <c r="D16" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="E16" t="s">
         <v>42</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
@@ -3187,7 +3211,7 @@
         <v>46</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
@@ -3207,7 +3231,7 @@
         <v>50</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
@@ -3227,7 +3251,7 @@
         <v>53</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -3247,7 +3271,7 @@
         <v>56</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3267,7 +3291,7 @@
         <v>59</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
@@ -3287,7 +3311,7 @@
         <v>62</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -3307,7 +3331,7 @@
         <v>64</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
@@ -3327,7 +3351,7 @@
         <v>66</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
@@ -3347,7 +3371,7 @@
         <v>69</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3367,7 +3391,7 @@
         <v>71</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
@@ -3387,7 +3411,7 @@
         <v>74</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
@@ -3407,7 +3431,7 @@
         <v>77</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
@@ -3427,7 +3451,7 @@
         <v>80</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -3553,7 +3577,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADD646AB-7E33-9A4A-B118-8FB38A78DA5A}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="64.83203125" bestFit="1" customWidth="1"/>
@@ -3572,116 +3596,118 @@
         <v>1</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="E1" s="11" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>366</v>
+        <v>403</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>365</v>
+        <v>404</v>
       </c>
       <c r="C2" s="11">
         <v>2026</v>
       </c>
       <c r="D2" s="14">
+        <v>46199</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>406</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>363</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>362</v>
+      </c>
+      <c r="C3" s="11">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="14">
         <v>46128</v>
       </c>
-      <c r="E2" s="11" t="s">
-        <v>397</v>
-      </c>
-      <c r="F2" s="11" t="s">
+      <c r="E3" s="11" t="s">
         <v>393</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>284</v>
-      </c>
-      <c r="B3" t="s">
-        <v>286</v>
-      </c>
-      <c r="C3" s="11">
-        <v>2025</v>
-      </c>
-      <c r="D3" s="14">
-        <v>45735</v>
-      </c>
-      <c r="E3" t="s">
-        <v>322</v>
-      </c>
-      <c r="F3" t="s">
-        <v>394</v>
+      <c r="F3" s="11" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>324</v>
+        <v>282</v>
       </c>
       <c r="B4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C4" s="11">
         <v>2025</v>
       </c>
       <c r="D4" s="14">
-        <v>45795</v>
+        <v>45735</v>
       </c>
       <c r="E4" t="s">
-        <v>395</v>
+        <v>320</v>
       </c>
       <c r="F4" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>323</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>302</v>
+        <v>322</v>
+      </c>
+      <c r="B5" t="s">
+        <v>285</v>
       </c>
       <c r="C5" s="11">
         <v>2025</v>
       </c>
       <c r="D5" s="14">
+        <v>45795</v>
+      </c>
+      <c r="E5" t="s">
+        <v>391</v>
+      </c>
+      <c r="F5" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>321</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="C6" s="11">
+        <v>2025</v>
+      </c>
+      <c r="D6" s="14">
         <v>45789</v>
       </c>
-      <c r="E5" t="s">
-        <v>396</v>
-      </c>
-      <c r="F5" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A6" s="11" t="s">
-        <v>109</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>87</v>
-      </c>
-      <c r="C6" s="11">
-        <v>2024</v>
-      </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11" t="s">
-        <v>110</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>393</v>
+      <c r="E6" t="s">
+        <v>392</v>
+      </c>
+      <c r="F6" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>87</v>
@@ -3691,51 +3717,51 @@
       </c>
       <c r="D7" s="11"/>
       <c r="E7" s="11" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="C8" s="11">
-        <v>2021</v>
+        <v>2024</v>
       </c>
       <c r="D8" s="11"/>
       <c r="E8" s="11" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C9" s="11">
-        <v>2019</v>
+        <v>2021</v>
       </c>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B10" s="11" t="s">
         <v>117</v>
@@ -3745,33 +3771,33 @@
       </c>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="11" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>87</v>
+        <v>117</v>
       </c>
       <c r="C11" s="11">
         <v>2019</v>
       </c>
       <c r="D11" s="11"/>
       <c r="E11" s="11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B12" s="11" t="s">
         <v>87</v>
@@ -3781,15 +3807,15 @@
       </c>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B13" s="11" t="s">
         <v>87</v>
@@ -3799,15 +3825,15 @@
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>398</v>
+        <v>124</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="11" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B14" s="11" t="s">
         <v>87</v>
@@ -3817,53 +3843,71 @@
       </c>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>127</v>
+        <v>394</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B15" s="11" t="s">
         <v>87</v>
       </c>
       <c r="C15" s="11">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D15" s="11"/>
       <c r="E15" s="11" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>117</v>
+        <v>87</v>
       </c>
       <c r="C16" s="11">
         <v>2018</v>
       </c>
       <c r="D16" s="11"/>
       <c r="E16" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="11">
+        <v>2018</v>
+      </c>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11" t="s">
         <v>131</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C17" s="6"/>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="F17" s="11" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="C18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C19" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3872,7 +3916,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FD52188-922E-CF44-BFD0-18928D31283D}">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.5" customWidth="1"/>
@@ -3888,10 +3932,10 @@
         <v>23</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="E1" s="4" t="s">
         <v>24</v>
@@ -3903,15 +3947,15 @@
         <v>4</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C2" s="12">
         <v>46279</v>
@@ -3920,108 +3964,108 @@
         <v>46281</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="11" t="s">
-        <v>359</v>
+        <v>396</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C3" s="12">
-        <v>46147</v>
+        <v>46224</v>
       </c>
       <c r="D3" s="12">
-        <v>46150</v>
+        <v>46226</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>180</v>
+        <v>361</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>191</v>
+        <v>397</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>361</v>
+        <v>398</v>
       </c>
       <c r="H3" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>194</v>
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="11" t="s">
+        <v>402</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
       <c r="C4" s="12">
-        <v>45960</v>
+        <v>46199</v>
       </c>
       <c r="D4" s="12">
-        <v>45961</v>
+        <v>46199</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>180</v>
+        <v>29</v>
       </c>
       <c r="F4" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G4" t="s">
-        <v>340</v>
+      <c r="G4" s="11" t="s">
+        <v>405</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>184</v>
+        <v>389</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="11" t="s">
+        <v>356</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
       <c r="C5" s="12">
-        <v>45735</v>
+        <v>46147</v>
       </c>
       <c r="D5" s="12">
-        <v>45736</v>
+        <v>46150</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>180</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>331</v>
-      </c>
-      <c r="G5" t="s">
-        <v>341</v>
+        <v>191</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>358</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>338</v>
+        <v>194</v>
       </c>
       <c r="B6" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C6" s="12">
-        <v>45943</v>
+        <v>45960</v>
       </c>
       <c r="D6" s="12">
-        <v>45944</v>
+        <v>45961</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>180</v>
@@ -4030,242 +4074,254 @@
         <v>8</v>
       </c>
       <c r="G6" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="H6" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>339</v>
+        <v>184</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C7" s="12">
-        <v>45838</v>
+        <v>45735</v>
       </c>
       <c r="D7" s="12">
-        <v>45841</v>
+        <v>45736</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>180</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>8</v>
+        <v>329</v>
       </c>
       <c r="G7" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>325</v>
+        <v>336</v>
       </c>
       <c r="B8" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C8" s="12">
-        <v>45831</v>
+        <v>45943</v>
       </c>
       <c r="D8" s="12">
-        <v>45835</v>
+        <v>45944</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>202</v>
+        <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>344</v>
+        <v>340</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>225</v>
+        <v>337</v>
       </c>
       <c r="B9" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C9" s="12">
-        <v>45783</v>
+        <v>45838</v>
       </c>
       <c r="D9" s="12">
-        <v>45783</v>
+        <v>45841</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>29</v>
+        <v>180</v>
       </c>
       <c r="F9" s="11" t="s">
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>345</v>
+        <v>341</v>
       </c>
       <c r="H9" s="11" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="10" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>288</v>
+        <v>323</v>
       </c>
       <c r="B10" s="15" t="s">
         <v>262</v>
       </c>
       <c r="C10" s="12">
+        <v>45831</v>
+      </c>
+      <c r="D10" s="12">
+        <v>45835</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>181</v>
+      </c>
+      <c r="F10" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="G10" t="s">
+        <v>342</v>
+      </c>
+      <c r="H10" s="11" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>225</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C11" s="12">
+        <v>45783</v>
+      </c>
+      <c r="D11" s="12">
+        <v>45783</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>343</v>
+      </c>
+      <c r="H11" s="11" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="11" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>286</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C12" s="12">
         <v>45889</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D12" s="12">
         <v>45889</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E12" s="11" t="s">
         <v>180</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F12" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="G10" t="s">
-        <v>346</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>211</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E11" t="s">
-        <v>329</v>
-      </c>
-      <c r="F11" t="s">
-        <v>213</v>
-      </c>
-      <c r="G11" t="s">
-        <v>244</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>190</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" t="s">
-        <v>181</v>
-      </c>
-      <c r="F12" t="s">
-        <v>192</v>
-      </c>
       <c r="G12" t="s">
-        <v>242</v>
+        <v>344</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>181</v>
+        <v>327</v>
       </c>
       <c r="F13" t="s">
-        <v>41</v>
+        <v>213</v>
       </c>
       <c r="G13" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="H13" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="E14" t="s">
         <v>181</v>
       </c>
       <c r="F14" t="s">
-        <v>8</v>
+        <v>192</v>
       </c>
       <c r="G14" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="H14" s="11" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>228</v>
+        <v>194</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>210</v>
+        <v>37</v>
       </c>
       <c r="E15" t="s">
-        <v>29</v>
+        <v>181</v>
       </c>
       <c r="F15" t="s">
-        <v>188</v>
+        <v>41</v>
       </c>
       <c r="G15" t="s">
-        <v>229</v>
+        <v>240</v>
       </c>
       <c r="H15" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>186</v>
+        <v>212</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>210</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>29</v>
+        <v>181</v>
       </c>
       <c r="F16" t="s">
-        <v>188</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>183</v>
-      </c>
-      <c r="B17" s="6">
-        <v>2021</v>
+        <v>228</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="E17" t="s">
         <v>29</v>
@@ -4274,135 +4330,135 @@
         <v>188</v>
       </c>
       <c r="G17" t="s">
-        <v>185</v>
+        <v>229</v>
       </c>
       <c r="H17" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>184</v>
-      </c>
-      <c r="B18" s="6">
-        <v>2021</v>
+        <v>186</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>210</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="G18" t="s">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="H18" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B19" s="6">
         <v>2021</v>
       </c>
       <c r="E19" t="s">
-        <v>180</v>
+        <v>29</v>
       </c>
       <c r="F19" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="G19" t="s">
-        <v>239</v>
+        <v>185</v>
       </c>
       <c r="H19" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B20" s="6">
         <v>2021</v>
       </c>
       <c r="E20" t="s">
-        <v>329</v>
+        <v>180</v>
       </c>
       <c r="F20" t="s">
         <v>191</v>
       </c>
       <c r="G20" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="H20" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B21" s="6">
         <v>2021</v>
       </c>
       <c r="E21" t="s">
-        <v>29</v>
+        <v>180</v>
       </c>
       <c r="F21" t="s">
         <v>191</v>
       </c>
       <c r="G21" t="s">
-        <v>209</v>
+        <v>239</v>
       </c>
       <c r="H21" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B22" s="6">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E22" t="s">
-        <v>180</v>
+        <v>327</v>
       </c>
       <c r="F22" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="G22" t="s">
-        <v>189</v>
+        <v>230</v>
       </c>
       <c r="H22" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="B23" s="6">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="E23" t="s">
-        <v>181</v>
+        <v>29</v>
       </c>
       <c r="F23" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G23" t="s">
-        <v>241</v>
+        <v>209</v>
       </c>
       <c r="H23" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>238</v>
+        <v>186</v>
       </c>
       <c r="B24" s="6">
         <v>2020</v>
@@ -4411,38 +4467,38 @@
         <v>180</v>
       </c>
       <c r="F24" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="G24" t="s">
-        <v>239</v>
+        <v>189</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B25" s="6">
         <v>2020</v>
       </c>
       <c r="E25" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F25" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G25" t="s">
-        <v>232</v>
+        <v>241</v>
       </c>
       <c r="H25" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>200</v>
+        <v>238</v>
       </c>
       <c r="B26" s="6">
         <v>2020</v>
@@ -4454,75 +4510,75 @@
         <v>191</v>
       </c>
       <c r="G26" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H26" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B27" s="6">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E27" t="s">
-        <v>329</v>
+        <v>180</v>
       </c>
       <c r="F27" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G27" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="H27" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B28" s="6">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="E28" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F28" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="G28" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H28" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B29" s="6">
         <v>2019</v>
       </c>
       <c r="E29" t="s">
-        <v>207</v>
+        <v>327</v>
       </c>
       <c r="F29" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="G29" t="s">
-        <v>206</v>
+        <v>231</v>
       </c>
       <c r="H29" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B30" s="6">
         <v>2019</v>
@@ -4531,58 +4587,58 @@
         <v>181</v>
       </c>
       <c r="F30" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
       <c r="G30" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B31" s="6">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E31" t="s">
-        <v>180</v>
+        <v>207</v>
       </c>
       <c r="F31" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G31" t="s">
-        <v>237</v>
+        <v>206</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B32" s="6">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E32" t="s">
-        <v>330</v>
+        <v>181</v>
       </c>
       <c r="F32" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G32" t="s">
-        <v>208</v>
+        <v>235</v>
       </c>
       <c r="H32" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B33" s="6">
         <v>2018</v>
@@ -4591,42 +4647,74 @@
         <v>180</v>
       </c>
       <c r="F33" t="s">
-        <v>8</v>
+        <v>204</v>
       </c>
       <c r="G33" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B34" s="6">
         <v>2018</v>
       </c>
       <c r="E34" t="s">
+        <v>328</v>
+      </c>
+      <c r="F34" t="s">
+        <v>203</v>
+      </c>
+      <c r="G34" t="s">
+        <v>208</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>200</v>
+      </c>
+      <c r="B35" s="6">
+        <v>2018</v>
+      </c>
+      <c r="E35" t="s">
         <v>180</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F35" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" t="s">
+        <v>236</v>
+      </c>
+      <c r="H35" s="11" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>201</v>
+      </c>
+      <c r="B36" s="6">
+        <v>2018</v>
+      </c>
+      <c r="E36" t="s">
+        <v>180</v>
+      </c>
+      <c r="F36" t="s">
         <v>205</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G36" t="s">
         <v>234</v>
       </c>
-      <c r="H34" s="11" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E38" s="6"/>
-      <c r="F38" s="6"/>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E39" s="6"/>
-      <c r="F39" s="6"/>
+      <c r="H36" s="11" t="s">
+        <v>390</v>
+      </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="E40" s="6"/>
@@ -4692,9 +4780,17 @@
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
     </row>
+    <row r="56" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E56" s="6"/>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="5:6" x14ac:dyDescent="0.2">
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A17:G34">
-    <sortCondition descending="1" ref="B1:B34"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A19:G36">
+    <sortCondition descending="1" ref="B1:B36"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4729,19 +4825,19 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="B2" s="11">
         <v>2025</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -4912,70 +5008,70 @@
         <v>149</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="F1" s="13" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C2">
         <v>2026</v>
       </c>
       <c r="D2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="E2" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F2" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B3" t="s">
-        <v>356</v>
+        <v>400</v>
       </c>
       <c r="C3">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D3" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E3" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="F3" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B4" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C4">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="E4" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
       <c r="F4" t="s">
-        <v>394</v>
+        <v>389</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4989,18 +5085,18 @@
         <v>2025</v>
       </c>
       <c r="D5" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="E5" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
       <c r="F5" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B6" t="s">
         <v>152</v>
@@ -5009,13 +5105,13 @@
         <v>2023</v>
       </c>
       <c r="D6" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E6" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
       <c r="F6" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -5029,13 +5125,13 @@
         <v>2023</v>
       </c>
       <c r="D7" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E7" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
       <c r="F7" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -5049,13 +5145,13 @@
         <v>2023</v>
       </c>
       <c r="D8" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E8" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
       <c r="F8" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -5069,13 +5165,13 @@
         <v>2022</v>
       </c>
       <c r="D9" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="E9" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
       <c r="F9" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -5089,13 +5185,13 @@
         <v>2021</v>
       </c>
       <c r="D10" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E10" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
       <c r="F10" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>